<commit_message>
Mise à jour Creation_TableAssociation
</commit_message>
<xml_diff>
--- a/input/DM_Excel/Creation_TableAssociation.xlsx
+++ b/input/DM_Excel/Creation_TableAssociation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ANS\NOS\GitHub\PJ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ANS\NOS\GitHub\DM_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB11F1A-CCF1-4104-8B41-F5372A127BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C27AB12-7792-44A8-9ED0-BB3AE272D7BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="750" windowWidth="29040" windowHeight="17520" xr2:uid="{8A89A1CA-4901-4EFB-B2E4-1C13CDDECCD6}"/>
   </bookViews>
@@ -347,7 +347,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -370,13 +370,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -407,9 +444,6 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -449,6 +483,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -812,258 +855,258 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.4">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
     </row>
     <row r="9" spans="1:6" ht="15.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="11" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="14"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="29"/>
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="14"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="29"/>
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:6" ht="34.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="14" t="s">
         <v>49</v>
       </c>
       <c r="F15" s="9"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="16"/>
-      <c r="B16" s="17" t="s">
+      <c r="A16" s="15"/>
+      <c r="B16" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="14"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="13"/>
       <c r="F16" s="10"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="19"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="14"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="19"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="14"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="13"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="19"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="14"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="13"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="19"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="14"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="13"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="19"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="14"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="13"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="19"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="14"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="13"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="14"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="29"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="14"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="29"/>
     </row>
     <row r="28" spans="1:4" ht="34.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="B28" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="14" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" s="16"/>
-      <c r="B29" s="17" t="s">
+      <c r="A29" s="15"/>
+      <c r="B29" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="18"/>
-      <c r="D29" s="14"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="13"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="19"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="14"/>
+      <c r="A30" s="18"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="13"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="19"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="14"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="13"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="19"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="14"/>
+      <c r="A32" s="18"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="13"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" s="19"/>
-      <c r="B33" s="17"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="14"/>
+      <c r="A33" s="18"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="13"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" s="19"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="14"/>
+      <c r="A34" s="18"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="13"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" s="19"/>
-      <c r="B35" s="17"/>
-      <c r="C35" s="19"/>
-      <c r="D35" s="14"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="13"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" s="20" t="s">
+      <c r="A37" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="16">
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A3:B3"/>
@@ -1076,6 +1119,10 @@
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>

</xml_diff>